<commit_message>
feat: Actual Payment manual input (non-KB/FP), Rebate % hide for non-KB/FP, per-user filter memory, Rebate default 10, import template Actual Payment col
</commit_message>
<xml_diff>
--- a/data/PL output/PL map.xlsx
+++ b/data/PL output/PL map.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C102"/>
+  <dimension ref="A1:C106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -543,7 +543,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Rex14</t>
+          <t>Rex14-QMB</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -560,7 +560,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Rex16</t>
+          <t>Rex16-QMB</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -572,12 +572,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>MCLAREN</t>
+          <t>Roz14-QMB</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>MCLAREN</t>
+          <t>Roz14-QMB</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -589,182 +589,182 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>VARCOLAC</t>
+          <t>Oaken14-QMB</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>VARCOLAC</t>
+          <t>Oaken14-QMB</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>TA</t>
+          <t>6U</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Vlad/Vlad6U Early Closed FY25Q3</t>
+          <t>Oaken16-QMB</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Vlad Early closed</t>
+          <t>Oaken16-QMB</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>KV</t>
+          <t>6U</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Vlad/Vlad6U Early Closed FY25Q3</t>
+          <t>Broncos-TH</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Vlad6U Early closed</t>
+          <t>Broncos-TH</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>KV</t>
+          <t>TA</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Andaman/Andaman6U Early Closed Fy25Q3</t>
+          <t>MCLAREN</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Andaman Early closed</t>
+          <t>MCLAREN</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>KV</t>
+          <t>AN</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Andaman/Andaman6U Early Closed Fy25Q3</t>
+          <t>VARCOLAC</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Andaman6U Early closed</t>
+          <t>VARCOLAC</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>KV</t>
+          <t>TA</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>NITTANY</t>
+          <t>Vlad/Vlad6U Early Closed FY25Q3</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>NITTANY</t>
+          <t>Vlad Early closed</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>M8</t>
+          <t>KV</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>WILLIE</t>
+          <t>Vlad/Vlad6U Early Closed FY25Q3</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>WILLIE</t>
+          <t>Vlad6U Early closed</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>M8</t>
+          <t>KV</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>LAPRASA/LAPRASI</t>
+          <t>Andaman/Andaman6U Early Closed Fy25Q3</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>LAPRASA</t>
+          <t>Andaman Early closed</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>M5</t>
+          <t>KV</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>LAPRASA/LAPRASI</t>
+          <t>Andaman/Andaman6U Early Closed Fy25Q3</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>LAPRASI</t>
+          <t>Andaman6U Early closed</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>M5</t>
+          <t>KV</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>MARVELA</t>
+          <t>NITTANY</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>MARVELA</t>
+          <t>NITTANY</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>DG</t>
+          <t>M8</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>HAYDEN</t>
+          <t>WILLIE</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>HAYDEN</t>
+          <t>WILLIE</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -776,136 +776,136 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Maldives/Maldives6u/MaldivesR6u Early closed FY25Q3</t>
+          <t>LAPRASA/LAPRASI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Maldives Early closed</t>
+          <t>LAPRASA</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>6U</t>
+          <t>M5</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Maldives/Maldives6u/MaldivesR6u Early closed FY25Q3</t>
+          <t>LAPRASA/LAPRASI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Maldives6u Early closed</t>
+          <t>LAPRASI</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>6U</t>
+          <t>M5</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Maldives/Maldives6u/MaldivesR6u Early closed FY25Q3</t>
+          <t>MARVELA</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>MaldivesR6u Early closed</t>
+          <t>MARVELA</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>6U</t>
+          <t>DG</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>SANDWALKER</t>
+          <t>HAYDEN</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>SANDWALKER</t>
+          <t>HAYDEN</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>M0</t>
+          <t>M8</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>CARM24ADG/CARM24IDG/CARMB24A/CARMB24I</t>
+          <t>Maldives/Maldives6u/MaldivesR6u Early closed FY25Q3</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>CARM24ADG</t>
+          <t>Maldives Early closed</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>1M</t>
+          <t>6U</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>CARM24ADG/CARM24IDG/CARMB24A/CARMB24I</t>
+          <t>Maldives/Maldives6u/MaldivesR6u Early closed FY25Q3</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>CARM24IDG</t>
+          <t>Maldives6u Early closed</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>1M</t>
+          <t>6U</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>CARM24ADG/CARM24IDG/CARMB24A/CARMB24I</t>
+          <t>Maldives/Maldives6u/MaldivesR6u Early closed FY25Q3</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>CARMB24A</t>
+          <t>MaldivesR6u Early closed</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>1M</t>
+          <t>6U</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>CARM24ADG/CARM24IDG/CARMB24A/CARMB24I</t>
+          <t>SANDWALKER</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>CARMB24I</t>
+          <t>SANDWALKER</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>1M</t>
+          <t>M0</t>
         </is>
       </c>
     </row>
@@ -922,7 +922,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>DG</t>
+          <t>1M</t>
         </is>
       </c>
     </row>
@@ -939,7 +939,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>DG</t>
+          <t>1M</t>
         </is>
       </c>
     </row>
@@ -956,7 +956,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>DG</t>
+          <t>1M</t>
         </is>
       </c>
     </row>
@@ -973,87 +973,87 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>DG</t>
+          <t>1M</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>TUFFY</t>
+          <t>CARM24ADG/CARM24IDG/CARMB24A/CARMB24I</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>TUFFY</t>
+          <t>CARM24ADG</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>KV</t>
+          <t>DG</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>PIKEWKS</t>
+          <t>CARM24ADG/CARM24IDG/CARMB24A/CARMB24I</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>PIKEWKS</t>
+          <t>CARM24IDG</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>5X</t>
+          <t>DG</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>MALDIVES/MALDIVES6U/MALDIVESR6U</t>
+          <t>CARM24ADG/CARM24IDG/CARMB24A/CARMB24I</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>MALDIVES</t>
+          <t>CARMB24A</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>KV</t>
+          <t>DG</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>MALDIVES/MALDIVES6U/MALDIVESR6U</t>
+          <t>CARM24ADG/CARM24IDG/CARMB24A/CARMB24I</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>MALDIVES6U</t>
+          <t>CARMB24I</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>KV</t>
+          <t>DG</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>MALDIVES/MALDIVES6U/MALDIVESR6U</t>
+          <t>TUFFY</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>MALDIVESR6U</t>
+          <t>TUFFY</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1065,80 +1065,80 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>GOLDY</t>
+          <t>PIKEWKS</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>GOLDY</t>
+          <t>PIKEWKS</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>M8</t>
+          <t>5X</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>ARIZONA</t>
+          <t>MALDIVES/MALDIVES6U/MALDIVESR6U</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>ARIZONA</t>
+          <t>MALDIVES</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>6U</t>
+          <t>KV</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>ANDAZ</t>
+          <t>MALDIVES/MALDIVES6U/MALDIVESR6U</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>ANDAZ</t>
+          <t>MALDIVES6U</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>M8</t>
+          <t>KV</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>TESTUDO</t>
+          <t>MALDIVES/MALDIVES6U/MALDIVESR6U</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>TESTUDO</t>
+          <t>MALDIVESR6U</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>M8</t>
+          <t>KV</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>HERBIE</t>
+          <t>GOLDY</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>HERBIE</t>
+          <t>GOLDY</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1150,68 +1150,68 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>WARG13/WARG14/WARG14L/WARG16</t>
+          <t>ARIZONA</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>WARG13</t>
+          <t>ARIZONA</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>AN</t>
+          <t>6U</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>WARG13/WARG14/WARG14L/WARG16</t>
+          <t>ANDAZ</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>WARG14</t>
+          <t>ANDAZ</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>AN</t>
+          <t>M8</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>WARG13/WARG14/WARG14L/WARG16</t>
+          <t>TESTUDO</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>WARG14L</t>
+          <t>TESTUDO</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>AN</t>
+          <t>M8</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>WARG13/WARG14/WARG14L/WARG16</t>
+          <t>HERBIE</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>WARG16</t>
+          <t>HERBIE</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>AN</t>
+          <t>M8</t>
         </is>
       </c>
     </row>
@@ -1228,7 +1228,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>M0</t>
+          <t>AN</t>
         </is>
       </c>
     </row>
@@ -1245,7 +1245,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>M0</t>
+          <t>AN</t>
         </is>
       </c>
     </row>
@@ -1262,7 +1262,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>M0</t>
+          <t>AN</t>
         </is>
       </c>
     </row>
@@ -1279,279 +1279,279 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>M0</t>
+          <t>AN</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>GRAND</t>
+          <t>WARG13/WARG14/WARG14L/WARG16</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>GRAND</t>
+          <t>WARG13</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>M8</t>
+          <t>M0</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>REGENCY</t>
+          <t>WARG13/WARG14/WARG14L/WARG16</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>REGENCY</t>
+          <t>WARG14</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>M8</t>
+          <t>M0</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>PARK</t>
+          <t>WARG13/WARG14/WARG14L/WARG16</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>PARK</t>
+          <t>WARG14L</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>M8</t>
+          <t>M0</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>BIGRED</t>
+          <t>WARG13/WARG14/WARG14L/WARG16</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>BIGRED</t>
+          <t>WARG16</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>M7</t>
+          <t>M0</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>RITCHIE</t>
+          <t>GRAND</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>RITCHIE</t>
+          <t>GRAND</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>M7</t>
+          <t>M8</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>ROAREE</t>
+          <t>REGENCY</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>ROAREE</t>
+          <t>REGENCY</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>M7</t>
+          <t>M8</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>BAYMAXW14/BAYMAXW16</t>
+          <t>PARK</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>BAYMAXW14</t>
+          <t>PARK</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>AN</t>
+          <t>M8</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>BAYMAXW14/BAYMAXW16</t>
+          <t>BIGRED</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>BAYMAXW16</t>
+          <t>BIGRED</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>AN</t>
+          <t>M7</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>RIESLING</t>
+          <t>RITCHIE</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>RIESLING</t>
+          <t>RITCHIE</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>KV</t>
+          <t>M7</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Warg14-IMP</t>
+          <t>ROAREE</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Warg14</t>
+          <t>ROAREE</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>AN</t>
+          <t>M7</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>QUAKER</t>
+          <t>BAYMAXW14/BAYMAXW16</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>QUAKER</t>
+          <t>BAYMAXW14</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>M7</t>
+          <t>AN</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>SPARTY</t>
+          <t>BAYMAXW14/BAYMAXW16</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>SPARTY</t>
+          <t>BAYMAXW16</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>M8</t>
+          <t>AN</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>LUISA13/LUISA14/LUISA16/LUISAW14</t>
+          <t>RIESLING</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>LUISA13</t>
+          <t>RIESLING</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>IK</t>
+          <t>KV</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>LUISA13/LUISA14/LUISA16/LUISAW14</t>
+          <t>Warg14-IMP</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>LUISA14</t>
+          <t>Warg14-IMP</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>IK</t>
+          <t>AN</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>LUISA13/LUISA14/LUISA16/LUISAW14</t>
+          <t>QUAKER</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>LUISA16</t>
+          <t>QUAKER</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>IK</t>
+          <t>M7</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>LUISA13/LUISA14/LUISA16/LUISAW14</t>
+          <t>SPARTY</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>LUISAW14</t>
+          <t>SPARTY</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>IK</t>
+          <t>M8</t>
         </is>
       </c>
     </row>
@@ -1568,7 +1568,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>AN</t>
+          <t>IK</t>
         </is>
       </c>
     </row>
@@ -1585,7 +1585,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>AN</t>
+          <t>IK</t>
         </is>
       </c>
     </row>
@@ -1602,7 +1602,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>AN</t>
+          <t>IK</t>
         </is>
       </c>
     </row>
@@ -1619,70 +1619,70 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>AN</t>
+          <t>IK</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>THOMPSON</t>
+          <t>LUISA13/LUISA14/LUISA16/LUISAW14</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>THOMPSON</t>
+          <t>LUISA13</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>M8</t>
+          <t>AN</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Ernesto-TH</t>
+          <t>LUISA13/LUISA14/LUISA16/LUISAW14</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Ernesto</t>
+          <t>LUISA14</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>M0</t>
+          <t>AN</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>HIMALAYAN</t>
+          <t>LUISA13/LUISA14/LUISA16/LUISAW14</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>HIMALAYAN</t>
+          <t>LUISA16</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>G7</t>
+          <t>AN</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>KRAKEN13</t>
+          <t>LUISA13/LUISA14/LUISA16/LUISAW14</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>KRAKEN13</t>
+          <t>LUISAW14</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -1694,12 +1694,12 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>OSKI</t>
+          <t>THOMPSON</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>OSKI</t>
+          <t>THOMPSON</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -1711,46 +1711,46 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>RAMESES6U</t>
+          <t>Ernesto-TH</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>RAMESES6U</t>
+          <t>Ernesto-TH</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>6U</t>
+          <t>M0</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Luisa-IMP</t>
+          <t>HIMALAYAN</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Luisa</t>
+          <t>HIMALAYAN</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>IK</t>
+          <t>G7</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Luisa-IMP</t>
+          <t>KRAKEN13</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Luisa</t>
+          <t>KRAKEN13</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -1762,182 +1762,182 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Baymax W-IMP</t>
+          <t>OSKI</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Baymax</t>
+          <t>OSKI</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>AN</t>
+          <t>M8</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>HYATT</t>
+          <t>RAMESES6U</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>HYATT</t>
+          <t>RAMESES6U</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>M8</t>
+          <t>6U</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>ANDAZAN/ANDAZAN8C</t>
+          <t>Luisa-IMP</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>ANDAZAN</t>
+          <t>Luisa-IMP</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>M0</t>
+          <t>IK</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>ANDAZAN/ANDAZAN8C</t>
+          <t>Luisa-IMP</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>ANDAZAN8C</t>
+          <t>Luisa-IMP</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>M0</t>
+          <t>AN</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>FREDDO</t>
+          <t>Baymax W-IMP</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>FREDDO</t>
+          <t>Baymax</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>GA</t>
+          <t>AN</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>RADIOHEAD</t>
+          <t>HYATT</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>RADIOHEAD</t>
+          <t>HYATT</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>M1</t>
+          <t>M8</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>LONGHORNZ</t>
+          <t>ANDAZAN/ANDAZAN8C</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>LONGHORNZ</t>
+          <t>ANDAZAN</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>IK</t>
+          <t>M0</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>SOLITAIREZ</t>
+          <t>ANDAZAN/ANDAZAN8C</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>SOLITAIREZ</t>
+          <t>ANDAZAN8C</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>IL</t>
+          <t>M0</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>ERNESTO</t>
+          <t>FREDDO</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>ERNESTO</t>
+          <t>FREDDO</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>M0</t>
+          <t>GA</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>PAN14</t>
+          <t>RADIOHEAD</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>PAN14</t>
+          <t>RADIOHEAD</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>6U</t>
+          <t>M1</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Longhornz-QMB</t>
+          <t>LONGHORNZ</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Longhornz</t>
+          <t>LONGHORNZ</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -1949,46 +1949,46 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>NANTUCKET 1.0</t>
+          <t>SOLITAIREZ</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>NANTUCKET</t>
+          <t>SOLITAIREZ</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>IQ</t>
+          <t>IL</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>DEMACIAZHAN</t>
+          <t>ERNESTO</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>DEMACIAZHAN</t>
+          <t>ERNESTO</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>DG</t>
+          <t>M0</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>RamesesR6U-ITH</t>
+          <t>PAN14</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>RamesesR6U</t>
+          <t>PAN14</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -2000,151 +2000,219 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>RAMESESR6U</t>
+          <t>Longhornz-QMB</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>RAMESESR6U</t>
+          <t>Longhornz-QMB</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>6U</t>
+          <t>IK</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>BAYMAX14/BAYMAX16</t>
+          <t>NANTUCKET 1.0</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>BAYMAX14</t>
+          <t>NANTUCKET</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>AN</t>
+          <t>IQ</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>BAYMAX14/BAYMAX16</t>
+          <t>DEMACIAZHAN</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>BAYMAX16</t>
+          <t>DEMACIAZHAN</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>AN</t>
+          <t>DG</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>BURMILLA</t>
+          <t>RamesesR6U-ITH</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>BURMILLA</t>
+          <t>RamesesR6U-ITH</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>G7</t>
+          <t>6U</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Burmilla-QMB</t>
+          <t>RAMESESR6U</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Burmilla</t>
+          <t>RAMESESR6U</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>G7</t>
+          <t>6U</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Bobcats-TH</t>
+          <t>BAYMAX14/BAYMAX16</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Bobcats</t>
+          <t>BAYMAX14</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>TA</t>
+          <t>AN</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>BOBCATS</t>
+          <t>BAYMAX14/BAYMAX16</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>BOBCATS</t>
+          <t>BAYMAX16</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>TA</t>
+          <t>AN</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>BAYMAX13/BAYMAX13X</t>
+          <t>BURMILLA</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>BAYMAX13</t>
+          <t>BURMILLA</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>AN</t>
+          <t>G7</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
+          <t>Burmilla-QMB</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Burmilla-QMB</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>G7</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Bobcats-TH</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Bobcats-TH</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>TA</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>BOBCATS</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>BOBCATS</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>TA</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
           <t>BAYMAX13/BAYMAX13X</t>
         </is>
       </c>
-      <c r="B102" t="inlineStr">
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>BAYMAX13</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>AN</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>BAYMAX13/BAYMAX13X</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
         <is>
           <t>BAYMAX13X</t>
         </is>
       </c>
-      <c r="C102" t="inlineStr">
+      <c r="C106" t="inlineStr">
         <is>
           <t>AN</t>
         </is>
@@ -2405,13 +2473,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4B8B104D-011B-472A-BE41-E496D6B6CE51}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{69CCCF77-1068-4B1B-B59D-D1416721A007}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{797D0AFB-14FB-484A-A043-6C153549E742}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C41C722E-77C4-44FD-9B8C-811AF725949D}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BBCCF700-EE12-4656-8ED3-758E07E70742}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E6739112-44DA-4AC1-9422-F05A8A6C8E5F}"/>
 </file>
</xml_diff>